<commit_message>
Corrige CI: converte xlsx antes do pipeline e corrige dados fake
</commit_message>
<xml_diff>
--- a/data/raw_fake/clientes.xlsx
+++ b/data/raw_fake/clientes.xlsx
@@ -478,7 +478,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ID100000</t>
+          <t>ID599291</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -488,7 +488,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ID100000</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -644,7 +644,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ID100001</t>
+          <t>ID786493</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -654,7 +654,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ID100001</t>
+          <t>ID352622</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -747,7 +747,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ID100002</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -757,7 +757,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ID100002</t>
+          <t>ID747843</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -850,7 +850,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ID100003</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -860,7 +860,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ID100003</t>
+          <t>ID547824</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -953,7 +953,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ID100004</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -963,7 +963,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ID100004</t>
+          <t>ID309811</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1056,7 +1056,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ID100005</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1066,7 +1066,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ID100005</t>
+          <t>ID675810</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1159,7 +1159,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ID100006</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1169,7 +1169,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ID100006</t>
+          <t>ID528435</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1262,7 +1262,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ID100007</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ID100007</t>
+          <t>ID523373</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1365,7 +1365,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ID100008</t>
+          <t>ID389860</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ID100008</t>
+          <t>ID929234</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1468,7 +1468,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ID100009</t>
+          <t>ID967817</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1478,7 +1478,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ID100009</t>
+          <t>ID636285</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1571,7 +1571,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ID100010</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1581,7 +1581,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ID100010</t>
+          <t>ID628668</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1674,7 +1674,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ID100011</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1684,7 +1684,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ID100011</t>
+          <t>ID231870</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1777,7 +1777,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ID100012</t>
+          <t>ID516205</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1787,7 +1787,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ID100012</t>
+          <t>ID204260</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1880,7 +1880,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ID100013</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ID100013</t>
+          <t>ID127724</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1983,7 +1983,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ID100014</t>
+          <t>ID402572</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1993,7 +1993,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ID100014</t>
+          <t>ID352526</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2086,7 +2086,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ID100015</t>
+          <t>ID231391</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ID100015</t>
+          <t>ID814297</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2189,7 +2189,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ID100016</t>
+          <t>ID153010</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2199,7 +2199,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ID100016</t>
+          <t>ID538181</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2292,7 +2292,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ID100017</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2302,7 +2302,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ID100017</t>
+          <t>ID199172</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2395,7 +2395,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ID100018</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2405,7 +2405,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>ID100018</t>
+          <t>ID535609</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2498,7 +2498,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ID100019</t>
+          <t>ID424337</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ID100019</t>
+          <t>ID699601</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2601,7 +2601,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ID100020</t>
+          <t>ID766894</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2611,7 +2611,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ID100020</t>
+          <t>ID185253</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2708,7 +2708,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ID100021</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2718,7 +2718,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ID100021</t>
+          <t>ID257641</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2811,7 +2811,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ID100022</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2821,7 +2821,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ID100022</t>
+          <t>ID874417</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2914,7 +2914,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ID100023</t>
+          <t>ID393612</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2924,7 +2924,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ID100023</t>
+          <t>ID235046</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -3017,7 +3017,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ID100024</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ID100024</t>
+          <t>ID489744</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -3120,7 +3120,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ID100025</t>
+          <t>ID102849</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3130,7 +3130,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ID100025</t>
+          <t>ID107148</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -3223,7 +3223,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ID100026</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ID100026</t>
+          <t>ID936006</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -3326,7 +3326,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ID100027</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3336,7 +3336,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ID100027</t>
+          <t>ID275618</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -3429,7 +3429,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ID100028</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3439,7 +3439,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ID100028</t>
+          <t>ID505935</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3532,7 +3532,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ID100029</t>
+          <t>ID944525</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3542,7 +3542,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ID100029</t>
+          <t>ID392446</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -3635,7 +3635,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ID100030</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3645,7 +3645,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ID100030</t>
+          <t>ID643048</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3738,7 +3738,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ID100031</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -3748,7 +3748,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ID100031</t>
+          <t>ID678968</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -3841,7 +3841,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ID100032</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -3851,7 +3851,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ID100032</t>
+          <t>ID513460</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -3944,7 +3944,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ID100033</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3954,7 +3954,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ID100033</t>
+          <t>ID442477</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -4047,7 +4047,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ID100034</t>
+          <t>ID147465</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -4057,7 +4057,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ID100034</t>
+          <t>ID768967</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -4150,7 +4150,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ID100035</t>
+          <t>ID449567</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -4160,7 +4160,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ID100035</t>
+          <t>ID393004</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -4253,7 +4253,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ID100036</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -4263,7 +4263,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ID100036</t>
+          <t>ID590835</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -4356,7 +4356,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ID100037</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -4366,7 +4366,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ID100037</t>
+          <t>ID376547</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -4459,7 +4459,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ID100038</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -4469,7 +4469,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ID100038</t>
+          <t>ID492763</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -4562,7 +4562,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ID100039</t>
+          <t>ID642195</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -4572,7 +4572,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>ID100039</t>
+          <t>ID126534</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -4665,7 +4665,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ID100040</t>
+          <t>ID215013</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -4675,7 +4675,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>ID100040</t>
+          <t>ID217189</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -4772,7 +4772,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ID100041</t>
+          <t>ID566121</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -4782,7 +4782,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>ID100041</t>
+          <t>ID909320</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -4879,7 +4879,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ID100042</t>
+          <t>ID556889</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -4889,7 +4889,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>ID100042</t>
+          <t>ID239732</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -4982,7 +4982,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ID100043</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -4992,7 +4992,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>ID100043</t>
+          <t>ID467904</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -5085,7 +5085,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ID100044</t>
+          <t>ID145590</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -5095,7 +5095,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>ID100044</t>
+          <t>ID579459</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -5188,7 +5188,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>ID100045</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -5198,7 +5198,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ID100045</t>
+          <t>ID637603</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -5291,7 +5291,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>ID100046</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -5301,7 +5301,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ID100046</t>
+          <t>ID825951</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -5394,7 +5394,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ID100047</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -5404,7 +5404,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>ID100047</t>
+          <t>ID370425</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -5497,7 +5497,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>ID100048</t>
+          <t>ID198994</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -5507,7 +5507,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>ID100048</t>
+          <t>ID514042</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -5604,7 +5604,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>ID100049</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -5614,7 +5614,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>ID100049</t>
+          <t>ID199298</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -5707,7 +5707,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ID100050</t>
+          <t>ID149699</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -5717,7 +5717,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ID100050</t>
+          <t>ID407948</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -5814,7 +5814,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ID100051</t>
+          <t>ID145590</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -5824,7 +5824,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ID100051</t>
+          <t>ID173048</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -5921,7 +5921,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ID100052</t>
+          <t>ID969868</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -5931,7 +5931,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>ID100052</t>
+          <t>ID312822</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -6024,7 +6024,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>ID100053</t>
+          <t>ID842947</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -6034,7 +6034,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>ID100053</t>
+          <t>ID135199</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -6131,7 +6131,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ID100054</t>
+          <t>ID173048</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -6141,7 +6141,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>ID100054</t>
+          <t>ID220835</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -6238,7 +6238,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ID100055</t>
+          <t>ID890012</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -6248,7 +6248,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>ID100055</t>
+          <t>ID164346</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -6341,7 +6341,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>ID100056</t>
+          <t>ID204722</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -6351,7 +6351,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>ID100056</t>
+          <t>ID411310</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -6444,7 +6444,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ID100057</t>
+          <t>ID145590</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -6454,7 +6454,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>ID100057</t>
+          <t>ID786493</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -6551,7 +6551,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>ID100058</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -6561,7 +6561,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>ID100058</t>
+          <t>ID309050</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -6654,7 +6654,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ID100059</t>
+          <t>ID556889</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>ID100059</t>
+          <t>ID859333</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -6757,7 +6757,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>ID100060</t>
+          <t>ID215013</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -6767,7 +6767,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>ID100060</t>
+          <t>ID750511</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -6864,7 +6864,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>ID100061</t>
+          <t>ID217189</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -6874,7 +6874,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>ID100061</t>
+          <t>ID634724</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -6971,7 +6971,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ID100062</t>
+          <t>ID215013</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -6981,7 +6981,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>ID100062</t>
+          <t>ID472737</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -7078,7 +7078,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>ID100063</t>
+          <t>ID423950</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -7088,7 +7088,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>ID100063</t>
+          <t>ID229319</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -7181,7 +7181,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ID100064</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -7191,7 +7191,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>ID100064</t>
+          <t>ID530946</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -7284,7 +7284,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>ID100065</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -7294,7 +7294,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>ID100065</t>
+          <t>ID438763</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -7387,7 +7387,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>ID100066</t>
+          <t>ID949476</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -7397,7 +7397,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>ID100066</t>
+          <t>ID453768</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -7490,7 +7490,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ID100067</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -7500,7 +7500,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>ID100067</t>
+          <t>ID631563</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -7593,7 +7593,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>ID100068</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -7603,7 +7603,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>ID100068</t>
+          <t>ID536365</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -7696,7 +7696,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>ID100069</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -7706,7 +7706,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>ID100069</t>
+          <t>ID997731</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -7799,7 +7799,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>ID100070</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -7809,7 +7809,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>ID100070</t>
+          <t>ID328445</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -7902,7 +7902,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>ID100071</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -7912,7 +7912,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>ID100071</t>
+          <t>ID253273</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -8005,7 +8005,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>ID100072</t>
+          <t>ID653348</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -8015,7 +8015,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ID100072</t>
+          <t>ID772479</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8112,7 +8112,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>ID100073</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -8122,7 +8122,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ID100073</t>
+          <t>ID296561</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -8215,7 +8215,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>ID100074</t>
+          <t>ID220835</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -8225,7 +8225,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>ID100074</t>
+          <t>ID686441</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -8318,7 +8318,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>ID100075</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -8328,7 +8328,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>ID100075</t>
+          <t>ID102849</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -8425,7 +8425,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>ID100076</t>
+          <t>ID969868</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -8435,7 +8435,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>ID100076</t>
+          <t>ID230296</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -8528,7 +8528,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>ID100077</t>
+          <t>ID428193</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -8538,7 +8538,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>ID100077</t>
+          <t>ID903353</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -8631,7 +8631,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ID100078</t>
+          <t>ID786493</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -8641,7 +8641,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>ID100078</t>
+          <t>ID842391</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -8734,7 +8734,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>ID100079</t>
+          <t>ID879068</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -8744,7 +8744,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>ID100079</t>
+          <t>ID498945</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -8841,7 +8841,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>ID100080</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -8851,7 +8851,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>ID100080</t>
+          <t>ID327868</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -8944,7 +8944,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>ID100081</t>
+          <t>ID350076</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -8954,7 +8954,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>ID100081</t>
+          <t>ID390920</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -9051,7 +9051,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>ID100082</t>
+          <t>ID762632</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -9061,7 +9061,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>ID100082</t>
+          <t>ID989449</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -9154,7 +9154,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>ID100083</t>
+          <t>ID480080</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>ID100083</t>
+          <t>ID979276</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -9257,7 +9257,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>ID100084</t>
+          <t>ID777683</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -9267,7 +9267,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>ID100084</t>
+          <t>ID591588</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -9364,7 +9364,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>ID100085</t>
+          <t>ID969868</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -9374,7 +9374,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>ID100085</t>
+          <t>ID116738</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -9467,7 +9467,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>ID100086</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -9477,7 +9477,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>ID100086</t>
+          <t>ID212067</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -9570,7 +9570,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>ID100087</t>
+          <t>ID653348</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -9580,7 +9580,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>ID100087</t>
+          <t>ID418122</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -9677,7 +9677,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>ID100088</t>
+          <t>ID979276</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -9687,7 +9687,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>ID100088</t>
+          <t>ID336746</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -9780,7 +9780,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>ID100089</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -9790,7 +9790,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>ID100089</t>
+          <t>ID335092</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -9883,7 +9883,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>ID100090</t>
+          <t>ID541811</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -9893,7 +9893,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>ID100090</t>
+          <t>ID330039</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -9990,7 +9990,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>ID100091</t>
+          <t>ID253273</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -10000,7 +10000,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>ID100091</t>
+          <t>ID148542</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -10093,7 +10093,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>ID100092</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -10103,7 +10103,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>ID100092</t>
+          <t>ID202820</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -10196,7 +10196,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>ID100093</t>
+          <t>ID855706</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -10206,7 +10206,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>ID100093</t>
+          <t>ID393612</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -10303,7 +10303,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>ID100094</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -10313,7 +10313,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>ID100094</t>
+          <t>ID958763</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -10406,7 +10406,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>ID100095</t>
+          <t>ID813376</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -10416,7 +10416,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>ID100095</t>
+          <t>ID639961</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -10509,7 +10509,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>ID100096</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -10519,7 +10519,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>ID100096</t>
+          <t>ID690908</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -10612,7 +10612,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>ID100097</t>
+          <t>ID453331</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -10622,7 +10622,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>ID100097</t>
+          <t>ID812261</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -10715,7 +10715,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>ID100098</t>
+          <t>ID423950</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -10725,7 +10725,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>ID100098</t>
+          <t>ID166877</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -10818,7 +10818,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>ID100099</t>
+          <t>ID393612</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -10828,7 +10828,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>ID100099</t>
+          <t>ID657628</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -10925,7 +10925,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>ID100100</t>
+          <t>ID428193</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -10935,7 +10935,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>ID100100</t>
+          <t>ID235435</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -11028,7 +11028,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>ID100101</t>
+          <t>ID776479</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -11038,7 +11038,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>ID100101</t>
+          <t>ID402572</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -11131,7 +11131,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>ID100102</t>
+          <t>ID654802</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -11141,7 +11141,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>ID100102</t>
+          <t>ID944525</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -11238,7 +11238,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>ID100103</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -11248,7 +11248,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>ID100103</t>
+          <t>ID667062</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -11341,7 +11341,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>ID100104</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -11351,7 +11351,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>ID100104</t>
+          <t>ID645488</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -11444,7 +11444,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>ID100105</t>
+          <t>ID952126</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -11454,7 +11454,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>ID100105</t>
+          <t>ID879482</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -11551,7 +11551,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>ID100106</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -11561,7 +11561,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>ID100106</t>
+          <t>ID178718</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -11654,7 +11654,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>ID100107</t>
+          <t>ID350076</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -11664,7 +11664,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>ID100107</t>
+          <t>ID250625</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -11761,7 +11761,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>ID100108</t>
+          <t>ID198994</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -11771,7 +11771,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>ID100108</t>
+          <t>ID247359</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -11868,7 +11868,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>ID100109</t>
+          <t>ID424337</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -11878,7 +11878,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>ID100109</t>
+          <t>ID899639</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -11971,7 +11971,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>ID100110</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -11981,7 +11981,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>ID100110</t>
+          <t>ID989420</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -12074,7 +12074,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>ID100111</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -12084,7 +12084,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>ID100111</t>
+          <t>ID761503</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -12177,7 +12177,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>ID100112</t>
+          <t>ID428193</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -12187,7 +12187,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>ID100112</t>
+          <t>ID256668</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -12280,7 +12280,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>ID100113</t>
+          <t>ID897878</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -12290,7 +12290,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>ID100113</t>
+          <t>ID530755</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -12387,7 +12387,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>ID100114</t>
+          <t>ID663796</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -12397,7 +12397,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>ID100114</t>
+          <t>ID116719</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -12494,7 +12494,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>ID100115</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -12504,7 +12504,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>ID100115</t>
+          <t>ID967623</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -12597,7 +12597,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>ID100116</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -12607,7 +12607,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>ID100116</t>
+          <t>ID355774</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -12700,7 +12700,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>ID100117</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -12710,7 +12710,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>ID100117</t>
+          <t>ID674301</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -12803,7 +12803,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>ID100118</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -12813,7 +12813,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>ID100118</t>
+          <t>ID652939</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -12906,7 +12906,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>ID100119</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -12916,7 +12916,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>ID100119</t>
+          <t>ID749293</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -13009,7 +13009,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>ID100120</t>
+          <t>ID369023</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -13019,7 +13019,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>ID100120</t>
+          <t>ID447265</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -13116,7 +13116,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>ID100121</t>
+          <t>ID164346</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -13126,7 +13126,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>ID100121</t>
+          <t>ID561492</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -13219,7 +13219,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>ID100122</t>
+          <t>ID215013</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -13229,7 +13229,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>ID100122</t>
+          <t>ID996416</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -13326,7 +13326,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>ID100123</t>
+          <t>ID428193</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -13336,7 +13336,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>ID100123</t>
+          <t>ID731847</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -13429,7 +13429,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>ID100124</t>
+          <t>ID790961</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -13439,7 +13439,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>ID100124</t>
+          <t>ID876920</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -13532,7 +13532,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>ID100125</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -13542,7 +13542,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>ID100125</t>
+          <t>ID216599</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -13635,7 +13635,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>ID100126</t>
+          <t>ID786493</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -13645,7 +13645,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>ID100126</t>
+          <t>ID908555</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -13738,7 +13738,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>ID100127</t>
+          <t>ID147735</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -13748,7 +13748,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>ID100127</t>
+          <t>ID243075</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -13841,7 +13841,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>ID100128</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -13851,7 +13851,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>ID100128</t>
+          <t>ID147735</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -13948,7 +13948,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>ID100129</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -13958,7 +13958,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>ID100129</t>
+          <t>ID354774</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -14051,7 +14051,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>ID100130</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -14061,7 +14061,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>ID100130</t>
+          <t>ID389860</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -14154,7 +14154,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>ID100131</t>
+          <t>ID164346</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -14164,7 +14164,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>ID100131</t>
+          <t>ID772223</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -14257,7 +14257,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>ID100132</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -14267,7 +14267,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>ID100132</t>
+          <t>ID470812</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -14364,7 +14364,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>ID100133</t>
+          <t>ID145590</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -14374,7 +14374,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>ID100133</t>
+          <t>ID227545</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -14471,7 +14471,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>ID100134</t>
+          <t>ID786493</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -14481,7 +14481,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>ID100134</t>
+          <t>ID308342</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -14574,7 +14574,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>ID100135</t>
+          <t>ID428193</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -14584,7 +14584,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>ID100135</t>
+          <t>ID440333</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -14677,7 +14677,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>ID100136</t>
+          <t>ID145590</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -14687,7 +14687,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>ID100136</t>
+          <t>ID430391</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -14784,7 +14784,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>ID100137</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -14794,7 +14794,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>ID100137</t>
+          <t>ID648902</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -14887,7 +14887,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>ID100138</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -14897,7 +14897,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>ID100138</t>
+          <t>ID698727</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -14990,7 +14990,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>ID100139</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -15000,7 +15000,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>ID100139</t>
+          <t>ID725430</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -15093,7 +15093,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>ID100140</t>
+          <t>ID989449</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -15103,7 +15103,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>ID100140</t>
+          <t>ID151324</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -15196,7 +15196,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>ID100141</t>
+          <t>ID807818</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -15206,7 +15206,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>ID100141</t>
+          <t>ID919783</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -15299,7 +15299,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>ID100142</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -15309,7 +15309,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>ID100142</t>
+          <t>ID409516</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -15402,7 +15402,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>ID100143</t>
+          <t>ID556581</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -15412,7 +15412,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>ID100143</t>
+          <t>ID437678</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -15505,7 +15505,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>ID100144</t>
+          <t>ID657628</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -15515,7 +15515,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>ID100144</t>
+          <t>ID780193</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -15608,7 +15608,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>ID100145</t>
+          <t>ID790961</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -15618,7 +15618,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>ID100145</t>
+          <t>ID233297</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -15711,7 +15711,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>ID100146</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -15721,7 +15721,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>ID100146</t>
+          <t>ID206414</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -15814,7 +15814,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>ID100147</t>
+          <t>ID786493</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -15824,7 +15824,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>ID100147</t>
+          <t>ID889653</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -15921,7 +15921,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>ID100148</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -15931,7 +15931,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>ID100148</t>
+          <t>ID458327</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -16024,7 +16024,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>ID100149</t>
+          <t>ID766894</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -16034,7 +16034,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>ID100149</t>
+          <t>ID454194</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -16131,7 +16131,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>ID100150</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -16141,7 +16141,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>ID100150</t>
+          <t>ID185248</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -16234,7 +16234,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>ID100151</t>
+          <t>ID809821</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -16244,7 +16244,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>ID100151</t>
+          <t>ID145590</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -16341,7 +16341,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>ID100152</t>
+          <t>ID449567</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -16351,7 +16351,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>ID100152</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -16448,7 +16448,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>ID100153</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -16458,7 +16458,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>ID100153</t>
+          <t>ID288528</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -16551,7 +16551,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>ID100154</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -16561,7 +16561,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>ID100154</t>
+          <t>ID464297</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -16654,7 +16654,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>ID100155</t>
+          <t>ID393612</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -16664,7 +16664,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>ID100155</t>
+          <t>ID121223</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -16757,7 +16757,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>ID100156</t>
+          <t>ID217189</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -16767,7 +16767,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>ID100156</t>
+          <t>ID766034</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -16860,7 +16860,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>ID100157</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -16870,7 +16870,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>ID100157</t>
+          <t>ID285250</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -16963,7 +16963,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>ID100158</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -16973,7 +16973,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>ID100158</t>
+          <t>ID378405</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -17066,7 +17066,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>ID100159</t>
+          <t>ID428193</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -17076,7 +17076,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>ID100159</t>
+          <t>ID685124</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -17169,7 +17169,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>ID100160</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -17179,7 +17179,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>ID100160</t>
+          <t>ID450915</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -17272,7 +17272,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>ID100161</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -17282,7 +17282,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>ID100161</t>
+          <t>ID597926</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -17375,7 +17375,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>ID100162</t>
+          <t>ID449567</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -17385,7 +17385,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>ID100162</t>
+          <t>ID359926</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -17478,7 +17478,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>ID100163</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -17488,7 +17488,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>ID100163</t>
+          <t>ID784783</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -17581,7 +17581,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>ID100164</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -17591,7 +17591,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>ID100164</t>
+          <t>ID609226</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -17684,7 +17684,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>ID100165</t>
+          <t>ID147735</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -17694,7 +17694,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>ID100165</t>
+          <t>ID367740</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -17787,7 +17787,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>ID100166</t>
+          <t>ID428193</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -17797,7 +17797,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>ID100166</t>
+          <t>ID835254</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -17890,7 +17890,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>ID100167</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -17900,7 +17900,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>ID100167</t>
+          <t>ID850280</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -17993,7 +17993,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>ID100168</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -18003,7 +18003,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>ID100168</t>
+          <t>ID688574</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
@@ -18096,7 +18096,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>ID100169</t>
+          <t>ID350076</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -18106,7 +18106,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>ID100169</t>
+          <t>ID949476</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -18203,7 +18203,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>ID100170</t>
+          <t>ID217189</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -18213,7 +18213,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>ID100170</t>
+          <t>ID971511</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
@@ -18306,7 +18306,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>ID100171</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -18316,7 +18316,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>ID100171</t>
+          <t>ID333066</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -18409,7 +18409,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>ID100172</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -18419,7 +18419,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>ID100172</t>
+          <t>ID128482</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -18512,7 +18512,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>ID100173</t>
+          <t>ID653348</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -18522,7 +18522,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>ID100173</t>
+          <t>ID980646</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -18619,7 +18619,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>ID100174</t>
+          <t>ID215013</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -18629,7 +18629,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>ID100174</t>
+          <t>ID776479</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -18726,7 +18726,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>ID100175</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -18736,7 +18736,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>ID100175</t>
+          <t>ID658683</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -18829,7 +18829,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>ID100176</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -18839,7 +18839,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>ID100176</t>
+          <t>ID567729</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -18932,7 +18932,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>ID100177</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -18942,7 +18942,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>ID100177</t>
+          <t>ID423950</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -19035,7 +19035,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>ID100178</t>
+          <t>ID389541</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -19045,7 +19045,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>ID100178</t>
+          <t>ID739146</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -19138,7 +19138,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>ID100179</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
@@ -19148,7 +19148,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>ID100179</t>
+          <t>ID844951</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -19245,7 +19245,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>ID100180</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -19255,7 +19255,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>ID100180</t>
+          <t>ID858247</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
@@ -19348,7 +19348,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>ID100181</t>
+          <t>ID393612</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -19358,7 +19358,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>ID100181</t>
+          <t>ID249228</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -19455,7 +19455,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>ID100182</t>
+          <t>ID516205</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -19465,7 +19465,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>ID100182</t>
+          <t>ID675508</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -19558,7 +19558,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>ID100183</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -19568,7 +19568,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>ID100183</t>
+          <t>ID235077</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
@@ -19661,7 +19661,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>ID100184</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -19671,7 +19671,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>ID100184</t>
+          <t>ID759936</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -19764,7 +19764,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>ID100185</t>
+          <t>ID462960</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -19774,7 +19774,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>ID100185</t>
+          <t>ID126300</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
@@ -19871,7 +19871,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>ID100186</t>
+          <t>ID751203</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -19881,7 +19881,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>ID100186</t>
+          <t>ID454449</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">

</xml_diff>